<commit_message>
feat: AGENT admissions portal
</commit_message>
<xml_diff>
--- a/AGENT/data/admissions.xlsx
+++ b/AGENT/data/admissions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,11 +477,16 @@
           <t>final_merit_score</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>STU-419D76BE</t>
+          <t>STU-7F8550DC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -491,7 +496,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>talha.aslam@test.com</t>
+          <t>paperphilo4@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -517,19 +522,142 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Eligible</t>
+          <t>Admitted</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>The student's marks_percentage (85) is mathematically greater than or equal to the threshold for BS Software Engineering (</t>
+          <t>The student's marks_percentage (85) is mathematically greater than or equal to the threshold for BS Software Engineering (75%).</t>
         </is>
       </c>
       <c r="K2" t="n">
         <v>59</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>72</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>STU-354A9DA5</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Raja Ghayoor Khan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>raja.ghayoor@test.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0333-2223333</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BS Software Engineering</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>82</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>82204-0345881-5</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>23</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Admitted</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>The student's marks_percentage (82) is mathematically greater than the threshold for BS Software Engineering (75%).</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>51</v>
+      </c>
+      <c r="L3" t="n">
+        <v>66.5</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>STU-809142F8</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Aman Nadeem</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>aman.nadeem@test.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0333-4445555</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BS Software Engineering</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>79</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>82101-0675656-3</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>77</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Admitted</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>The student's marks_percentage (79) is mathematically greater than the threshold for BS Software Engineering (75%).</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>52</v>
+      </c>
+      <c r="L4" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>